<commit_message>
Remove 3 notas ja entregues (sem cadastro Parauapebas)
- Notas 2750680/2750344/2750986 (CODIGO 40931/40932/40933) baixadas
- Base: 159->156 recusas | R$ 8,29mi->8,27mi
- Sem reentrega: 131->128 | R$ 6,75mi->6,73mi
- MRO sem cadastro: 10->7 | Parauapebas fisico: 37->34
- Pedido MRO (78 cargas / R$ 2,63mi) inalterado
- Base tratada regenerada sem as 3

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PANxrCPXPZu6Z7SQtmhUMy
</commit_message>
<xml_diff>
--- a/apresentacoes/Devolucoes_Vale_tratada.xlsx
+++ b/apresentacoes/Devolucoes_Vale_tratada.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ160"/>
+  <dimension ref="A1:AJ157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -748,8 +748,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ2" t="b">
-        <v>0</v>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -898,8 +900,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ3" t="b">
-        <v>0</v>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1048,8 +1052,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ4" t="b">
-        <v>1</v>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1198,8 +1204,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ5" t="b">
-        <v>1</v>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1348,8 +1356,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ6" t="b">
-        <v>0</v>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1498,8 +1508,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ7" t="b">
-        <v>1</v>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1648,8 +1660,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ8" t="b">
-        <v>1</v>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1798,8 +1812,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ9" t="b">
-        <v>0</v>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1948,8 +1964,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ10" t="b">
-        <v>0</v>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -2098,8 +2116,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ11" t="b">
-        <v>0</v>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -2248,8 +2268,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ12" t="b">
-        <v>1</v>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2398,8 +2420,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ13" t="b">
-        <v>1</v>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2548,8 +2572,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ14" t="b">
-        <v>0</v>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2699,8 +2725,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ15" t="b">
-        <v>0</v>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -2850,8 +2878,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ16" t="b">
-        <v>0</v>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -3001,8 +3031,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ17" t="b">
-        <v>0</v>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -3152,8 +3184,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ18" t="b">
-        <v>0</v>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -3303,8 +3337,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ19" t="b">
-        <v>0</v>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -3454,8 +3490,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ20" t="b">
-        <v>0</v>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -3605,8 +3643,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ21" t="b">
-        <v>1</v>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -3756,8 +3796,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ22" t="b">
-        <v>1</v>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -3907,8 +3949,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ23" t="b">
-        <v>1</v>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -4056,8 +4100,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ24" t="b">
-        <v>1</v>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -4205,8 +4251,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ25" t="b">
-        <v>1</v>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -4356,8 +4404,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ26" t="b">
-        <v>1</v>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -4507,8 +4557,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ27" t="b">
-        <v>1</v>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -4658,8 +4710,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ28" t="b">
-        <v>1</v>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -4811,8 +4865,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ29" t="b">
-        <v>0</v>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -4962,8 +5018,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ30" t="b">
-        <v>1</v>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -5113,8 +5171,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ31" t="b">
-        <v>0</v>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -5262,8 +5322,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ32" t="b">
-        <v>0</v>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -5413,8 +5475,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ33" t="b">
-        <v>1</v>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -5564,8 +5628,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ34" t="b">
-        <v>0</v>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -5713,8 +5779,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ35" t="b">
-        <v>0</v>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -5862,8 +5930,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ36" t="b">
-        <v>0</v>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -6011,8 +6081,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ37" t="b">
-        <v>0</v>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -6162,8 +6234,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ38" t="b">
-        <v>1</v>
+      <c r="AJ38" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -6313,8 +6387,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ39" t="b">
-        <v>0</v>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -6464,8 +6540,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ40" t="b">
-        <v>0</v>
+      <c r="AJ40" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -6615,8 +6693,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ41" t="b">
-        <v>1</v>
+      <c r="AJ41" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -6766,8 +6846,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ42" t="b">
-        <v>0</v>
+      <c r="AJ42" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -6915,8 +6997,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ43" t="b">
-        <v>0</v>
+      <c r="AJ43" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -7064,8 +7148,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ44" t="b">
-        <v>0</v>
+      <c r="AJ44" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -7215,8 +7301,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ45" t="b">
-        <v>0</v>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -7364,8 +7452,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ46" t="b">
-        <v>0</v>
+      <c r="AJ46" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -7515,8 +7605,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ47" t="b">
-        <v>0</v>
+      <c r="AJ47" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -7666,8 +7758,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ48" t="b">
-        <v>0</v>
+      <c r="AJ48" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -7817,8 +7911,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ49" t="b">
-        <v>0</v>
+      <c r="AJ49" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -7966,8 +8062,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ50" t="b">
-        <v>0</v>
+      <c r="AJ50" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -8115,8 +8213,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ51" t="b">
-        <v>0</v>
+      <c r="AJ51" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -8266,8 +8366,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ52" t="b">
-        <v>0</v>
+      <c r="AJ52" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -8415,8 +8517,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ53" t="b">
-        <v>0</v>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -8566,8 +8670,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ54" t="b">
-        <v>0</v>
+      <c r="AJ54" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -8717,8 +8823,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ55" t="b">
-        <v>0</v>
+      <c r="AJ55" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -8866,8 +8974,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ56" t="b">
-        <v>0</v>
+      <c r="AJ56" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -9017,8 +9127,10 @@
           <t>UNENTEL SOLUCOES TECNOLOGICAS LTDA</t>
         </is>
       </c>
-      <c r="AJ57" t="b">
-        <v>0</v>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -9169,8 +9281,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ58" t="b">
-        <v>0</v>
+      <c r="AJ58" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -9291,8 +9405,10 @@
       </c>
       <c r="AH59" t="inlineStr"/>
       <c r="AI59" t="inlineStr"/>
-      <c r="AJ59" t="b">
-        <v>0</v>
+      <c r="AJ59" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -9441,8 +9557,10 @@
           <t>UNENTEL SOLUCOES TECNOLOGICAS LTDA</t>
         </is>
       </c>
-      <c r="AJ60" t="b">
-        <v>0</v>
+      <c r="AJ60" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -9592,8 +9710,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ61" t="b">
-        <v>0</v>
+      <c r="AJ61" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -9738,8 +9858,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ62" t="b">
-        <v>0</v>
+      <c r="AJ62" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -9885,8 +10007,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ63" t="b">
-        <v>0</v>
+      <c r="AJ63" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -10036,8 +10160,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ64" t="b">
-        <v>0</v>
+      <c r="AJ64" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -10187,8 +10313,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ65" t="b">
-        <v>0</v>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -10338,8 +10466,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ66" t="b">
-        <v>1</v>
+      <c r="AJ66" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -10487,8 +10617,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ67" t="b">
-        <v>1</v>
+      <c r="AJ67" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -10638,8 +10770,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ68" t="b">
-        <v>0</v>
+      <c r="AJ68" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -10789,8 +10923,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ69" t="b">
-        <v>0</v>
+      <c r="AJ69" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -10940,8 +11076,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ70" t="b">
-        <v>0</v>
+      <c r="AJ70" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -11091,8 +11229,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ71" t="b">
-        <v>0</v>
+      <c r="AJ71" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -11243,8 +11383,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ72" t="b">
-        <v>0</v>
+      <c r="AJ72" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -11394,8 +11536,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ73" t="b">
-        <v>0</v>
+      <c r="AJ73" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -11545,8 +11689,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ74" t="b">
-        <v>0</v>
+      <c r="AJ74" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -11696,8 +11842,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ75" t="b">
-        <v>1</v>
+      <c r="AJ75" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -11847,8 +11995,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ76" t="b">
-        <v>1</v>
+      <c r="AJ76" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -11998,8 +12148,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ77" t="b">
-        <v>0</v>
+      <c r="AJ77" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -12149,8 +12301,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ78" t="b">
-        <v>0</v>
+      <c r="AJ78" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -12300,8 +12454,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ79" t="b">
-        <v>0</v>
+      <c r="AJ79" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -12451,8 +12607,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ80" t="b">
-        <v>0</v>
+      <c r="AJ80" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -12604,8 +12762,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ81" t="b">
-        <v>0</v>
+      <c r="AJ81" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -12755,8 +12915,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ82" t="b">
-        <v>0</v>
+      <c r="AJ82" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -12906,8 +13068,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ83" t="b">
-        <v>0</v>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -13057,8 +13221,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ84" t="b">
-        <v>1</v>
+      <c r="AJ84" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -13208,8 +13374,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ85" t="b">
-        <v>0</v>
+      <c r="AJ85" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -13359,8 +13527,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ86" t="b">
-        <v>1</v>
+      <c r="AJ86" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -13510,8 +13680,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ87" t="b">
-        <v>1</v>
+      <c r="AJ87" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -13660,8 +13832,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ88" t="b">
-        <v>0</v>
+      <c r="AJ88" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -13811,8 +13985,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ89" t="b">
-        <v>0</v>
+      <c r="AJ89" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -13962,8 +14138,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ90" t="b">
-        <v>1</v>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -14113,8 +14291,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ91" t="b">
-        <v>0</v>
+      <c r="AJ91" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -14264,8 +14444,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ92" t="b">
-        <v>1</v>
+      <c r="AJ92" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -14415,8 +14597,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ93" t="b">
-        <v>1</v>
+      <c r="AJ93" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -14566,8 +14750,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ94" t="b">
-        <v>0</v>
+      <c r="AJ94" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -14717,8 +14903,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ95" t="b">
-        <v>0</v>
+      <c r="AJ95" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -14868,8 +15056,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ96" t="b">
-        <v>0</v>
+      <c r="AJ96" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -15018,8 +15208,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ97" t="b">
-        <v>0</v>
+      <c r="AJ97" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -15168,8 +15360,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ98" t="b">
-        <v>0</v>
+      <c r="AJ98" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -15318,8 +15512,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ99" t="b">
-        <v>0</v>
+      <c r="AJ99" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -15468,8 +15664,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ100" t="b">
-        <v>0</v>
+      <c r="AJ100" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -15618,8 +15816,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ101" t="b">
-        <v>0</v>
+      <c r="AJ101" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -15766,8 +15966,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ102" t="b">
-        <v>0</v>
+      <c r="AJ102" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -15916,8 +16118,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ103" t="b">
-        <v>0</v>
+      <c r="AJ103" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -16064,8 +16268,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ104" t="b">
-        <v>0</v>
+      <c r="AJ104" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -16214,8 +16420,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ105" t="b">
-        <v>0</v>
+      <c r="AJ105" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -16364,8 +16572,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ106" t="b">
-        <v>0</v>
+      <c r="AJ106" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -16514,8 +16724,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ107" t="b">
-        <v>0</v>
+      <c r="AJ107" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -16665,8 +16877,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ108" t="b">
-        <v>0</v>
+      <c r="AJ108" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -16785,8 +16999,10 @@
       </c>
       <c r="AH109" t="inlineStr"/>
       <c r="AI109" t="inlineStr"/>
-      <c r="AJ109" t="b">
-        <v>0</v>
+      <c r="AJ109" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -16932,8 +17148,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ110" t="b">
-        <v>0</v>
+      <c r="AJ110" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -17078,8 +17296,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ111" t="b">
-        <v>0</v>
+      <c r="AJ111" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -17201,8 +17421,10 @@
       </c>
       <c r="AH112" t="inlineStr"/>
       <c r="AI112" t="inlineStr"/>
-      <c r="AJ112" t="b">
-        <v>0</v>
+      <c r="AJ112" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -17351,8 +17573,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ113" t="b">
-        <v>0</v>
+      <c r="AJ113" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -17496,8 +17720,10 @@
           <t>TRANSPORTES DELLA VOLPE S A COMERCI</t>
         </is>
       </c>
-      <c r="AJ114" t="b">
-        <v>0</v>
+      <c r="AJ114" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="115">
@@ -17646,8 +17872,10 @@
           <t>ROLATEL COM DE ROLAMENTOS LT</t>
         </is>
       </c>
-      <c r="AJ115" t="b">
-        <v>0</v>
+      <c r="AJ115" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="116">
@@ -17796,8 +18024,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ116" t="b">
-        <v>0</v>
+      <c r="AJ116" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -17946,8 +18176,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ117" t="b">
-        <v>0</v>
+      <c r="AJ117" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -18096,8 +18328,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ118" t="b">
-        <v>0</v>
+      <c r="AJ118" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -18246,8 +18480,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ119" t="b">
-        <v>0</v>
+      <c r="AJ119" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -18396,8 +18632,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ120" t="b">
-        <v>0</v>
+      <c r="AJ120" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -18546,8 +18784,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ121" t="b">
-        <v>0</v>
+      <c r="AJ121" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -18696,8 +18936,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ122" t="b">
-        <v>0</v>
+      <c r="AJ122" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -18844,8 +19086,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ123" t="b">
-        <v>0</v>
+      <c r="AJ123" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -18994,8 +19238,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ124" t="b">
-        <v>0</v>
+      <c r="AJ124" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="125">
@@ -19114,8 +19360,10 @@
       </c>
       <c r="AH125" t="inlineStr"/>
       <c r="AI125" t="inlineStr"/>
-      <c r="AJ125" t="b">
-        <v>0</v>
+      <c r="AJ125" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -19256,8 +19504,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ126" t="b">
-        <v>0</v>
+      <c r="AJ126" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -19398,8 +19648,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ127" t="b">
-        <v>0</v>
+      <c r="AJ127" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="128">
@@ -19540,8 +19792,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ128" t="b">
-        <v>0</v>
+      <c r="AJ128" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="129">
@@ -19686,8 +19940,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ129" t="b">
-        <v>0</v>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="130">
@@ -19832,8 +20088,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ130" t="b">
-        <v>0</v>
+      <c r="AJ130" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="131">
@@ -19978,8 +20236,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ131" t="b">
-        <v>0</v>
+      <c r="AJ131" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="132">
@@ -20124,8 +20384,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ132" t="b">
-        <v>0</v>
+      <c r="AJ132" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="133">
@@ -20270,8 +20532,10 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ133" t="b">
-        <v>0</v>
+      <c r="AJ133" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="134">
@@ -20390,8 +20654,10 @@
       </c>
       <c r="AH134" t="inlineStr"/>
       <c r="AI134" t="inlineStr"/>
-      <c r="AJ134" t="b">
-        <v>0</v>
+      <c r="AJ134" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="135">
@@ -20510,8 +20776,10 @@
       </c>
       <c r="AH135" t="inlineStr"/>
       <c r="AI135" t="inlineStr"/>
-      <c r="AJ135" t="b">
-        <v>0</v>
+      <c r="AJ135" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -20630,8 +20898,10 @@
       </c>
       <c r="AH136" t="inlineStr"/>
       <c r="AI136" t="inlineStr"/>
-      <c r="AJ136" t="b">
-        <v>0</v>
+      <c r="AJ136" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -20750,18 +21020,20 @@
       </c>
       <c r="AH137" t="inlineStr"/>
       <c r="AI137" t="inlineStr"/>
-      <c r="AJ137" t="b">
-        <v>0</v>
+      <c r="AJ137" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>40931</t>
+          <t>40934</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>1370818</v>
+        <v>1345715</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -20774,7 +21046,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>2750680</v>
+        <v>19880</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
@@ -20799,7 +21071,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>35260557582793000111550010027506801600929056</t>
+          <t>35260504483719000181550010000198801014347341</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -20808,9 +21080,7 @@
         </is>
       </c>
       <c r="M138" t="inlineStr"/>
-      <c r="N138" t="n">
-        <v>4512827951</v>
-      </c>
+      <c r="N138" t="inlineStr"/>
       <c r="O138" t="inlineStr">
         <is>
           <t>PARAUAPEBAS</t>
@@ -20822,12 +21092,12 @@
       <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr">
         <is>
-          <t>FESTO  BRASIL LTDA</t>
+          <t>TRILHOS FERROVIARIOS LTDA</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>Unid.val.bloq. BR_CS.2238743 LINHA 10 BR</t>
+          <t>TRILHOS</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -20836,13 +21106,13 @@
         </is>
       </c>
       <c r="U138" t="n">
-        <v>300292000</v>
+        <v>300286000</v>
       </c>
       <c r="V138" t="n">
-        <v>6000177987</v>
+        <v>6000176656</v>
       </c>
       <c r="W138" s="1" t="n">
-        <v>46184</v>
+        <v>46182</v>
       </c>
       <c r="X138" t="inlineStr">
         <is>
@@ -20850,7 +21120,7 @@
         </is>
       </c>
       <c r="Y138" t="n">
-        <v>14274.96</v>
+        <v>6584.94</v>
       </c>
       <c r="Z138" t="inlineStr">
         <is>
@@ -20867,12 +21137,12 @@
       </c>
       <c r="AC138" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD138" t="inlineStr">
         <is>
-          <t>SEM CADASTRO.</t>
+          <t>DELVOVER AO FORNECEDOR, SEM ESPACO NO ARMAZEM. CLIENTE N?O RESPONDE.</t>
         </is>
       </c>
       <c r="AE138" t="inlineStr">
@@ -20900,18 +21170,20 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ138" t="b">
-        <v>0</v>
+      <c r="AJ138" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>40932</t>
+          <t>40935</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>1370767</v>
+        <v>1373906</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -20924,7 +21196,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>2750344</v>
+        <v>832161</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
@@ -20949,7 +21221,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>35260557582793000111550010027503441916055185</t>
+          <t>35260657599581000147550100008321611745969714</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -20959,7 +21231,7 @@
       </c>
       <c r="M139" t="inlineStr"/>
       <c r="N139" t="n">
-        <v>4513016302</v>
+        <v>4513157676</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -20972,12 +21244,12 @@
       <c r="Q139" t="inlineStr"/>
       <c r="R139" t="inlineStr">
         <is>
-          <t>FESTO  BRASIL LTDA</t>
+          <t>A.R.S. - INDUSTRIA E COMERCIO DE PA</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>ATUAD.SEMI-ROT DFPD-160-RP-90-RS60-F07e</t>
+          <t>PORCA SEXT M 16X2 CH 24 ZB-(4513157676)-</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -20986,7 +21258,7 @@
         </is>
       </c>
       <c r="U139" t="n">
-        <v>300290000</v>
+        <v>300292000</v>
       </c>
       <c r="V139" t="n">
         <v>6000177987</v>
@@ -21000,7 +21272,7 @@
         </is>
       </c>
       <c r="Y139" t="n">
-        <v>3111.84</v>
+        <v>2.09</v>
       </c>
       <c r="Z139" t="inlineStr">
         <is>
@@ -21050,18 +21322,20 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ139" t="b">
-        <v>0</v>
+      <c r="AJ139" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>40933</t>
+          <t>40936</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1370847</v>
+        <v>1373876</v>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -21074,7 +21348,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>2750986</v>
+        <v>832157</v>
       </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
@@ -21099,7 +21373,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>35260557582793000111550010027509861602346481</t>
+          <t>35260657599581000147550100008321571940142103</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -21109,7 +21383,7 @@
       </c>
       <c r="M140" t="inlineStr"/>
       <c r="N140" t="n">
-        <v>4513156749</v>
+        <v>4513156502</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -21122,12 +21396,12 @@
       <c r="Q140" t="inlineStr"/>
       <c r="R140" t="inlineStr">
         <is>
-          <t>FESTO  BRASIL LTDA</t>
+          <t>A.R.S. - INDUSTRIA E COMERCIO DE PA</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>TUBO FLEXIVEL PUN-10X1,5-BL LINHA 10</t>
+          <t>PA MAQ LENT 1/4-20X3/4 BC-(4513156502)-(</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -21150,7 +21424,7 @@
         </is>
       </c>
       <c r="Y140" t="n">
-        <v>1243.29</v>
+        <v>4.69</v>
       </c>
       <c r="Z140" t="inlineStr">
         <is>
@@ -21200,18 +21474,20 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ140" t="b">
-        <v>0</v>
+      <c r="AJ140" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>40934</t>
+          <t>40937</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1345715</v>
+        <v>1373877</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -21224,7 +21500,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>19880</v>
+        <v>832439</v>
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
@@ -21249,7 +21525,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>35260504483719000181550010000198801014347341</t>
+          <t>35260657599581000147550100008324391399034843</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -21258,7 +21534,9 @@
         </is>
       </c>
       <c r="M141" t="inlineStr"/>
-      <c r="N141" t="inlineStr"/>
+      <c r="N141" t="n">
+        <v>4513184897</v>
+      </c>
       <c r="O141" t="inlineStr">
         <is>
           <t>PARAUAPEBAS</t>
@@ -21270,12 +21548,12 @@
       <c r="Q141" t="inlineStr"/>
       <c r="R141" t="inlineStr">
         <is>
-          <t>TRILHOS FERROVIARIOS LTDA</t>
+          <t>A.R.S. - INDUSTRIA E COMERCIO DE PA</t>
         </is>
       </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t>TRILHOS</t>
+          <t>PORCA SEXT G.8 3/8-16-(4513184897)-(10)</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -21284,13 +21562,13 @@
         </is>
       </c>
       <c r="U141" t="n">
-        <v>300286000</v>
+        <v>300292000</v>
       </c>
       <c r="V141" t="n">
-        <v>6000176656</v>
+        <v>6000177987</v>
       </c>
       <c r="W141" s="1" t="n">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="X141" t="inlineStr">
         <is>
@@ -21298,7 +21576,7 @@
         </is>
       </c>
       <c r="Y141" t="n">
-        <v>6584.94</v>
+        <v>29.82</v>
       </c>
       <c r="Z141" t="inlineStr">
         <is>
@@ -21315,12 +21593,12 @@
       </c>
       <c r="AC141" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>.</t>
         </is>
       </c>
       <c r="AD141" t="inlineStr">
         <is>
-          <t>DELVOVER AO FORNECEDOR, SEM ESPACO NO ARMAZEM. CLIENTE N?O RESPONDE.</t>
+          <t>SEM CADASTRO.</t>
         </is>
       </c>
       <c r="AE141" t="inlineStr">
@@ -21348,18 +21626,20 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ141" t="b">
-        <v>0</v>
+      <c r="AJ141" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>40935</t>
+          <t>40938</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>1373906</v>
+        <v>1373725</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -21372,7 +21652,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>832161</v>
+        <v>832250</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -21397,7 +21677,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>35260657599581000147550100008321611745969714</t>
+          <t>35260657599581000147550100008322501737668575</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -21407,7 +21687,7 @@
       </c>
       <c r="M142" t="inlineStr"/>
       <c r="N142" t="n">
-        <v>4513157676</v>
+        <v>4513169468</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -21425,7 +21705,7 @@
       </c>
       <c r="S142" t="inlineStr">
         <is>
-          <t>PORCA SEXT M 16X2 CH 24 ZB-(4513157676)-</t>
+          <t>PA SEXT G.8 5/8-11X1.1/2  RI-(4513169468</t>
         </is>
       </c>
       <c r="T142" t="inlineStr">
@@ -21448,7 +21728,7 @@
         </is>
       </c>
       <c r="Y142" t="n">
-        <v>2.09</v>
+        <v>527.1799999999999</v>
       </c>
       <c r="Z142" t="inlineStr">
         <is>
@@ -21498,18 +21778,20 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ142" t="b">
-        <v>0</v>
+      <c r="AJ142" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>40936</t>
+          <t>40939</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>1373876</v>
+        <v>1373833</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -21522,7 +21804,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>832157</v>
+        <v>832328</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -21547,7 +21829,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>35260657599581000147550100008321571940142103</t>
+          <t>35260657599581000147550100008323281853076349</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -21557,7 +21839,7 @@
       </c>
       <c r="M143" t="inlineStr"/>
       <c r="N143" t="n">
-        <v>4513156502</v>
+        <v>4513176053</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -21575,7 +21857,7 @@
       </c>
       <c r="S143" t="inlineStr">
         <is>
-          <t>PA MAQ LENT 1/4-20X3/4 BC-(4513156502)-(</t>
+          <t>PORCA SEXT G.5 1/2-13 CH 3/4-(4513176053</t>
         </is>
       </c>
       <c r="T143" t="inlineStr">
@@ -21598,7 +21880,7 @@
         </is>
       </c>
       <c r="Y143" t="n">
-        <v>4.69</v>
+        <v>22.15</v>
       </c>
       <c r="Z143" t="inlineStr">
         <is>
@@ -21648,18 +21930,20 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ143" t="b">
-        <v>0</v>
+      <c r="AJ143" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>40937</t>
+          <t>40940</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>1373877</v>
+        <v>1373872</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -21672,7 +21956,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>832439</v>
+        <v>832297</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -21697,7 +21981,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>35260657599581000147550100008324391399034843</t>
+          <t>35260657599581000147550100008322971181221624</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -21707,7 +21991,7 @@
       </c>
       <c r="M144" t="inlineStr"/>
       <c r="N144" t="n">
-        <v>4513184897</v>
+        <v>4513176054</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -21725,7 +22009,7 @@
       </c>
       <c r="S144" t="inlineStr">
         <is>
-          <t>PORCA SEXT G.8 3/8-16-(4513184897)-(10)</t>
+          <t>PA SX G.5 1/2-13X1.1/2 RI ZB-(4513176054</t>
         </is>
       </c>
       <c r="T144" t="inlineStr">
@@ -21748,7 +22032,7 @@
         </is>
       </c>
       <c r="Y144" t="n">
-        <v>29.82</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="Z144" t="inlineStr">
         <is>
@@ -21798,18 +22082,20 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ144" t="b">
-        <v>0</v>
+      <c r="AJ144" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>40938</t>
+          <t>40941</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>1373725</v>
+        <v>1373907</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -21822,7 +22108,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>832250</v>
+        <v>832187</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -21847,7 +22133,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>35260657599581000147550100008322501737668575</t>
+          <t>35260657599581000147550100008321871884435103</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -21857,7 +22143,7 @@
       </c>
       <c r="M145" t="inlineStr"/>
       <c r="N145" t="n">
-        <v>4513169468</v>
+        <v>4513160425</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -21875,7 +22161,7 @@
       </c>
       <c r="S145" t="inlineStr">
         <is>
-          <t>PA SEXT G.8 5/8-11X1.1/2  RI-(4513169468</t>
+          <t>ARRUELA LISA DE ACO DIN 125 A M 18-(4513</t>
         </is>
       </c>
       <c r="T145" t="inlineStr">
@@ -21898,7 +22184,7 @@
         </is>
       </c>
       <c r="Y145" t="n">
-        <v>527.1799999999999</v>
+        <v>11.72</v>
       </c>
       <c r="Z145" t="inlineStr">
         <is>
@@ -21948,38 +22234,30 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ145" t="b">
-        <v>0</v>
+      <c r="AJ145" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>40939</t>
-        </is>
-      </c>
-      <c r="B146" t="n">
-        <v>1373833</v>
-      </c>
+          <t>40942</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr">
         <is>
           <t>Devolução</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>TDV São Paulo - SP</t>
-        </is>
-      </c>
+      <c r="D146" t="inlineStr"/>
       <c r="E146" t="n">
-        <v>832328</v>
+        <v>19878</v>
       </c>
       <c r="F146" t="inlineStr"/>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>FRACIONADO</t>
-        </is>
-      </c>
+      <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
           <t>PENDENTE</t>
@@ -21997,7 +22275,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>35260657599581000147550100008323281853076349</t>
+          <t>41260611340390000165550040000198781801155209</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -22006,9 +22284,7 @@
         </is>
       </c>
       <c r="M146" t="inlineStr"/>
-      <c r="N146" t="n">
-        <v>4513176053</v>
-      </c>
+      <c r="N146" t="inlineStr"/>
       <c r="O146" t="inlineStr">
         <is>
           <t>PARAUAPEBAS</t>
@@ -22020,35 +22296,25 @@
       <c r="Q146" t="inlineStr"/>
       <c r="R146" t="inlineStr">
         <is>
-          <t>A.R.S. - INDUSTRIA E COMERCIO DE PA</t>
-        </is>
-      </c>
-      <c r="S146" t="inlineStr">
-        <is>
-          <t>PORCA SEXT G.5 1/2-13 CH 3/4-(4513176053</t>
-        </is>
-      </c>
+          <t>ECOFIBRA INDUSTRIA E COMERCIO DE CO</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr"/>
       <c r="T146" t="inlineStr">
         <is>
           <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
         </is>
       </c>
-      <c r="U146" t="n">
-        <v>300292000</v>
-      </c>
-      <c r="V146" t="n">
-        <v>6000177987</v>
-      </c>
-      <c r="W146" s="1" t="n">
-        <v>46184</v>
-      </c>
+      <c r="U146" t="inlineStr"/>
+      <c r="V146" t="inlineStr"/>
+      <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
           <t>jsconceica</t>
         </is>
       </c>
       <c r="Y146" t="n">
-        <v>22.15</v>
+        <v>9584.99</v>
       </c>
       <c r="Z146" t="inlineStr">
         <is>
@@ -22065,12 +22331,12 @@
       </c>
       <c r="AC146" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="AD146" t="inlineStr">
         <is>
-          <t>SEM CADASTRO.</t>
+          <t>DESTINO DIVERGENTE</t>
         </is>
       </c>
       <c r="AE146" t="inlineStr">
@@ -22088,48 +22354,32 @@
           <t>PARAUAPEBAS</t>
         </is>
       </c>
-      <c r="AH146" t="inlineStr">
-        <is>
-          <t>VALE S.A.</t>
-        </is>
-      </c>
-      <c r="AI146" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AJ146" t="b">
-        <v>0</v>
+      <c r="AH146" t="inlineStr"/>
+      <c r="AI146" t="inlineStr"/>
+      <c r="AJ146" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>40940</t>
-        </is>
-      </c>
-      <c r="B147" t="n">
-        <v>1373872</v>
-      </c>
+          <t>40945</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr">
         <is>
           <t>Devolução</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>TDV São Paulo - SP</t>
-        </is>
-      </c>
+      <c r="D147" t="inlineStr"/>
       <c r="E147" t="n">
-        <v>832297</v>
+        <v>241473</v>
       </c>
       <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>FRACIONADO</t>
-        </is>
-      </c>
+      <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
           <t>PENDENTE</t>
@@ -22147,7 +22397,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>35260657599581000147550100008322971181221624</t>
+          <t>31260629799921000490550000002414731266548790</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
@@ -22156,49 +22406,37 @@
         </is>
       </c>
       <c r="M147" t="inlineStr"/>
-      <c r="N147" t="n">
-        <v>4513176054</v>
-      </c>
+      <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr">
         <is>
           <t>PARAUAPEBAS</t>
         </is>
       </c>
       <c r="P147" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="Q147" t="inlineStr"/>
       <c r="R147" t="inlineStr">
         <is>
-          <t>A.R.S. - INDUSTRIA E COMERCIO DE PA</t>
-        </is>
-      </c>
-      <c r="S147" t="inlineStr">
-        <is>
-          <t>PA SX G.5 1/2-13X1.1/2 RI ZB-(4513176054</t>
-        </is>
-      </c>
+          <t>ESAB IND E COM LTDA</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr"/>
       <c r="T147" t="inlineStr">
         <is>
           <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
         </is>
       </c>
-      <c r="U147" t="n">
-        <v>300292000</v>
-      </c>
-      <c r="V147" t="n">
-        <v>6000177987</v>
-      </c>
-      <c r="W147" s="1" t="n">
-        <v>46184</v>
-      </c>
+      <c r="U147" t="inlineStr"/>
+      <c r="V147" t="inlineStr"/>
+      <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
           <t>jsconceica</t>
         </is>
       </c>
       <c r="Y147" t="n">
-        <v>76.68000000000001</v>
+        <v>267397.26</v>
       </c>
       <c r="Z147" t="inlineStr">
         <is>
@@ -22211,16 +22449,16 @@
         </is>
       </c>
       <c r="AB147" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AC147" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="AD147" t="inlineStr">
         <is>
-          <t>SEM CADASTRO.</t>
+          <t>RECUSADO DEVIDO A DATA REMESSA SER FUTURA E SEM ALINHAMENTO DA VALE</t>
         </is>
       </c>
       <c r="AE147" t="inlineStr">
@@ -22238,48 +22476,32 @@
           <t>PARAUAPEBAS</t>
         </is>
       </c>
-      <c r="AH147" t="inlineStr">
-        <is>
-          <t>VALE S.A.</t>
-        </is>
-      </c>
-      <c r="AI147" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AJ147" t="b">
-        <v>0</v>
+      <c r="AH147" t="inlineStr"/>
+      <c r="AI147" t="inlineStr"/>
+      <c r="AJ147" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>40941</t>
-        </is>
-      </c>
-      <c r="B148" t="n">
-        <v>1373907</v>
-      </c>
+          <t>40946</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr">
         <is>
           <t>Devolução</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>TDV São Paulo - SP</t>
-        </is>
-      </c>
+      <c r="D148" t="inlineStr"/>
       <c r="E148" t="n">
-        <v>832187</v>
+        <v>241562</v>
       </c>
       <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>FRACIONADO</t>
-        </is>
-      </c>
+      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>PENDENTE</t>
@@ -22297,7 +22519,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>35260657599581000147550100008321871884435103</t>
+          <t>31260629799921000490550000002415621553848879</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
@@ -22306,49 +22528,37 @@
         </is>
       </c>
       <c r="M148" t="inlineStr"/>
-      <c r="N148" t="n">
-        <v>4513160425</v>
-      </c>
+      <c r="N148" t="inlineStr"/>
       <c r="O148" t="inlineStr">
         <is>
           <t>PARAUAPEBAS</t>
         </is>
       </c>
       <c r="P148" s="1" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="Q148" t="inlineStr"/>
       <c r="R148" t="inlineStr">
         <is>
-          <t>A.R.S. - INDUSTRIA E COMERCIO DE PA</t>
-        </is>
-      </c>
-      <c r="S148" t="inlineStr">
-        <is>
-          <t>ARRUELA LISA DE ACO DIN 125 A M 18-(4513</t>
-        </is>
-      </c>
+          <t>ESAB IND E COM LTDA</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr"/>
       <c r="T148" t="inlineStr">
         <is>
           <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
         </is>
       </c>
-      <c r="U148" t="n">
-        <v>300292000</v>
-      </c>
-      <c r="V148" t="n">
-        <v>6000177987</v>
-      </c>
-      <c r="W148" s="1" t="n">
-        <v>46184</v>
-      </c>
+      <c r="U148" t="inlineStr"/>
+      <c r="V148" t="inlineStr"/>
+      <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
           <t>jsconceica</t>
         </is>
       </c>
       <c r="Y148" t="n">
-        <v>11.72</v>
+        <v>178264.84</v>
       </c>
       <c r="Z148" t="inlineStr">
         <is>
@@ -22361,16 +22571,16 @@
         </is>
       </c>
       <c r="AB148" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AC148" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="AD148" t="inlineStr">
         <is>
-          <t>SEM CADASTRO.</t>
+          <t>RECUSADO DEVIDO A DATA REMESSA SER FUTURA E SEM ALINHAMENTO DA VALE</t>
         </is>
       </c>
       <c r="AE148" t="inlineStr">
@@ -22388,24 +22598,18 @@
           <t>PARAUAPEBAS</t>
         </is>
       </c>
-      <c r="AH148" t="inlineStr">
-        <is>
-          <t>VALE S.A.</t>
-        </is>
-      </c>
-      <c r="AI148" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AJ148" t="b">
-        <v>0</v>
+      <c r="AH148" t="inlineStr"/>
+      <c r="AI148" t="inlineStr"/>
+      <c r="AJ148" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>40942</t>
+          <t>40977</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
@@ -22416,7 +22620,7 @@
       </c>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="n">
-        <v>19878</v>
+        <v>857543</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
@@ -22437,7 +22641,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>41260611340390000165550040000198781801155209</t>
+          <t>35260600536772003249550010008575431753933138</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -22453,18 +22657,18 @@
         </is>
       </c>
       <c r="P149" s="1" t="n">
-        <v>46212</v>
+        <v>46217</v>
       </c>
       <c r="Q149" t="inlineStr"/>
       <c r="R149" t="inlineStr">
         <is>
-          <t>ECOFIBRA INDUSTRIA E COMERCIO DE CO</t>
+          <t>ECOLAB QUIMICA LTDA</t>
         </is>
       </c>
       <c r="S149" t="inlineStr"/>
       <c r="T149" t="inlineStr">
         <is>
-          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
+          <t>DEVOLUCAO INDEVIDA</t>
         </is>
       </c>
       <c r="U149" t="inlineStr"/>
@@ -22472,11 +22676,11 @@
       <c r="W149" t="inlineStr"/>
       <c r="X149" t="inlineStr">
         <is>
-          <t>jsconceica</t>
+          <t>erisoares</t>
         </is>
       </c>
       <c r="Y149" t="n">
-        <v>9584.99</v>
+        <v>215462.1</v>
       </c>
       <c r="Z149" t="inlineStr">
         <is>
@@ -22489,16 +22693,16 @@
         </is>
       </c>
       <c r="AB149" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="AC149" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD149" t="inlineStr">
         <is>
-          <t>DESTINO DIVERGENTE</t>
+          <t>MATERIAL DEVOLVIDO DEVIDO O CLIENTE ESTA SEM EQUIPAMENTO PRA DESCARREGAR, FAZER ALINHAMENTO COM CLIENTE E AREA.</t>
         </is>
       </c>
       <c r="AE149" t="inlineStr">
@@ -22508,7 +22712,7 @@
       </c>
       <c r="AF149" t="inlineStr">
         <is>
-          <t>9 - 12 Dias</t>
+          <t>0 - 8 Dias</t>
         </is>
       </c>
       <c r="AG149" t="inlineStr">
@@ -22518,28 +22722,40 @@
       </c>
       <c r="AH149" t="inlineStr"/>
       <c r="AI149" t="inlineStr"/>
-      <c r="AJ149" t="b">
-        <v>0</v>
+      <c r="AJ149" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>40945</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr"/>
+          <t>40219</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>1194154</v>
+      </c>
       <c r="C150" t="inlineStr">
         <is>
           <t>Devolução</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr"/>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>TDV Contagem MG</t>
+        </is>
+      </c>
       <c r="E150" t="n">
-        <v>241473</v>
+        <v>2593</v>
       </c>
       <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>FRACIONADO</t>
+        </is>
+      </c>
       <c r="H150" t="inlineStr">
         <is>
           <t>PENDENTE</t>
@@ -22547,17 +22763,17 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Parauapebas - PA</t>
+          <t>São Luíz - MA</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>31260629799921000490550000002414731266548790</t>
+          <t>31260415801747000116550030000025931705512966</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -22566,41 +22782,53 @@
         </is>
       </c>
       <c r="M150" t="inlineStr"/>
-      <c r="N150" t="inlineStr"/>
+      <c r="N150" t="n">
+        <v>4101104740</v>
+      </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="P150" s="1" t="n">
-        <v>46213</v>
+        <v>46136</v>
       </c>
       <c r="Q150" t="inlineStr"/>
       <c r="R150" t="inlineStr">
         <is>
-          <t>ESAB IND E COM LTDA</t>
-        </is>
-      </c>
-      <c r="S150" t="inlineStr"/>
+          <t>SEVEN SUPRIMENTOS INDUSTRIAIS LTDA</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>MANGUEIRA  P/COMPRESSOR PARAGUSO</t>
+        </is>
+      </c>
       <c r="T150" t="inlineStr">
         <is>
-          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
-        </is>
-      </c>
-      <c r="U150" t="inlineStr"/>
-      <c r="V150" t="inlineStr"/>
-      <c r="W150" t="inlineStr"/>
+          <t>NOTA FISCAL DIVERGENTE</t>
+        </is>
+      </c>
+      <c r="U150" t="n">
+        <v>300254000</v>
+      </c>
+      <c r="V150" t="n">
+        <v>6000153276</v>
+      </c>
+      <c r="W150" s="1" t="n">
+        <v>46122</v>
+      </c>
       <c r="X150" t="inlineStr">
         <is>
-          <t>jsconceica</t>
+          <t>dluz</t>
         </is>
       </c>
       <c r="Y150" t="n">
-        <v>267397.26</v>
+        <v>702.84</v>
       </c>
       <c r="Z150" t="inlineStr">
         <is>
-          <t>No Prazo</t>
+          <t>Atrasado</t>
         </is>
       </c>
       <c r="AA150" t="inlineStr">
@@ -22609,7 +22837,7 @@
         </is>
       </c>
       <c r="AB150" t="n">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="AC150" t="inlineStr">
         <is>
@@ -22618,48 +22846,68 @@
       </c>
       <c r="AD150" t="inlineStr">
         <is>
-          <t>RECUSADO DEVIDO A DATA REMESSA SER FUTURA E SEM ALINHAMENTO DA VALE</t>
+          <t>NF CONSTA DIVERGENCIA (INAPTA),NECESSARIO REGULARIZACAO DO XML. O FORNECEDOR DEVERA ABRIR CHAMADO NA FERRAMENTA V360</t>
         </is>
       </c>
       <c r="AE150" t="inlineStr">
         <is>
-          <t>IPATINGA/MG</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="AF150" t="inlineStr">
         <is>
-          <t>9 - 12 Dias</t>
+          <t>Acima de 12 Dias</t>
         </is>
       </c>
       <c r="AG150" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
-        </is>
-      </c>
-      <c r="AH150" t="inlineStr"/>
-      <c r="AI150" t="inlineStr"/>
-      <c r="AJ150" t="b">
-        <v>0</v>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AH150" t="inlineStr">
+        <is>
+          <t>VALE S A</t>
+        </is>
+      </c>
+      <c r="AI150" t="inlineStr">
+        <is>
+          <t>SEVEN SUPRIMENTOS INDUSTRIAIS LTDA</t>
+        </is>
+      </c>
+      <c r="AJ150" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>40946</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr"/>
+          <t>40547</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>392391</v>
+      </c>
       <c r="C151" t="inlineStr">
         <is>
           <t>Devolução</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>TDV São Luiz - MA</t>
+        </is>
+      </c>
       <c r="E151" t="n">
-        <v>241562</v>
+        <v>33540</v>
       </c>
       <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>FRACIONADO</t>
+        </is>
+      </c>
       <c r="H151" t="inlineStr">
         <is>
           <t>PENDENTE</t>
@@ -22667,17 +22915,17 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Parauapebas - PA</t>
+          <t>São Luíz - MA</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>31260629799921000490550000002415621553848879</t>
+          <t>35250500017952000118550010000335401611802796</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
@@ -22686,25 +22934,31 @@
         </is>
       </c>
       <c r="M151" t="inlineStr"/>
-      <c r="N151" t="inlineStr"/>
+      <c r="N151" t="n">
+        <v>4100989446</v>
+      </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="P151" s="1" t="n">
-        <v>46213</v>
+        <v>46171</v>
       </c>
       <c r="Q151" t="inlineStr"/>
       <c r="R151" t="inlineStr">
         <is>
-          <t>ESAB IND E COM LTDA</t>
-        </is>
-      </c>
-      <c r="S151" t="inlineStr"/>
+          <t>MOLYGRAFIT INDUSTRIA E COMERCIO LTD</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>SERVIÇO DE TRANSPORTE</t>
+        </is>
+      </c>
       <c r="T151" t="inlineStr">
         <is>
-          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
+          <t>NOTA FISCAL DIVERGENTE</t>
         </is>
       </c>
       <c r="U151" t="inlineStr"/>
@@ -22712,15 +22966,15 @@
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr">
         <is>
-          <t>jsconceica</t>
+          <t>dluz</t>
         </is>
       </c>
       <c r="Y151" t="n">
-        <v>178264.84</v>
+        <v>1029.23</v>
       </c>
       <c r="Z151" t="inlineStr">
         <is>
-          <t>No Prazo</t>
+          <t>Atrasado</t>
         </is>
       </c>
       <c r="AA151" t="inlineStr">
@@ -22729,7 +22983,7 @@
         </is>
       </c>
       <c r="AB151" t="n">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="AC151" t="inlineStr">
         <is>
@@ -22738,48 +22992,68 @@
       </c>
       <c r="AD151" t="inlineStr">
         <is>
-          <t>RECUSADO DEVIDO A DATA REMESSA SER FUTURA E SEM ALINHAMENTO DA VALE</t>
+          <t>FIZEMOS A TENTATIVA DE REENTREGA COM MESMA NF , JUNTO DA NF COMPLEMENTAR (33689) FONFORME TRATATIVAS , POREM NOTA CONTINUA INAPTA.</t>
         </is>
       </c>
       <c r="AE151" t="inlineStr">
         <is>
-          <t>IPATINGA/MG</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="AF151" t="inlineStr">
         <is>
-          <t>9 - 12 Dias</t>
+          <t>Acima de 12 Dias</t>
         </is>
       </c>
       <c r="AG151" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
-        </is>
-      </c>
-      <c r="AH151" t="inlineStr"/>
-      <c r="AI151" t="inlineStr"/>
-      <c r="AJ151" t="b">
-        <v>0</v>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AH151" t="inlineStr">
+        <is>
+          <t>VALE S A</t>
+        </is>
+      </c>
+      <c r="AI151" t="inlineStr">
+        <is>
+          <t>MOLYGRAFIT INDUSTRIA E COMERCIO LTD</t>
+        </is>
+      </c>
+      <c r="AJ151" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>40977</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr"/>
+          <t>40810</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1365998</v>
+      </c>
       <c r="C152" t="inlineStr">
         <is>
           <t>Devolução</t>
         </is>
       </c>
-      <c r="D152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>TDV Contagem MG</t>
+        </is>
+      </c>
       <c r="E152" t="n">
-        <v>857543</v>
+        <v>8466</v>
       </c>
       <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>FRACIONADO</t>
+        </is>
+      </c>
       <c r="H152" t="inlineStr">
         <is>
           <t>PENDENTE</t>
@@ -22787,17 +23061,17 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Parauapebas - PA</t>
+          <t>São Luíz - MA</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>35260600536772003249550010008575431753933138</t>
+          <t>31260343711951000505550010000084661325509470</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -22809,38 +23083,48 @@
       <c r="N152" t="inlineStr"/>
       <c r="O152" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="P152" s="1" t="n">
-        <v>46217</v>
+        <v>46196</v>
       </c>
       <c r="Q152" t="inlineStr"/>
       <c r="R152" t="inlineStr">
         <is>
-          <t>ECOLAB QUIMICA LTDA</t>
-        </is>
-      </c>
-      <c r="S152" t="inlineStr"/>
+          <t>FLSMIDTH INDUSTRIAL SOLUTIONS LTDA</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>PARTES</t>
+        </is>
+      </c>
       <c r="T152" t="inlineStr">
         <is>
-          <t>DEVOLUCAO INDEVIDA</t>
-        </is>
-      </c>
-      <c r="U152" t="inlineStr"/>
-      <c r="V152" t="inlineStr"/>
-      <c r="W152" t="inlineStr"/>
+          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
+        </is>
+      </c>
+      <c r="U152" t="n">
+        <v>300292000</v>
+      </c>
+      <c r="V152" t="n">
+        <v>6000181717</v>
+      </c>
+      <c r="W152" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="X152" t="inlineStr">
         <is>
-          <t>erisoares</t>
+          <t>proliveira</t>
         </is>
       </c>
       <c r="Y152" t="n">
-        <v>215462.1</v>
+        <v>1281886.36</v>
       </c>
       <c r="Z152" t="inlineStr">
         <is>
-          <t>No Prazo</t>
+          <t>Atrasado</t>
         </is>
       </c>
       <c r="AA152" t="inlineStr">
@@ -22849,47 +23133,57 @@
         </is>
       </c>
       <c r="AB152" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="AC152" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="AD152" t="inlineStr">
         <is>
-          <t>MATERIAL DEVOLVIDO DEVIDO O CLIENTE ESTA SEM EQUIPAMENTO PRA DESCARREGAR, FAZER ALINHAMENTO COM CLIENTE E AREA.</t>
+          <t>O FORNECEDOR DEVERA ABRIR CHAMADO NA FERRAMENTA V360</t>
         </is>
       </c>
       <c r="AE152" t="inlineStr">
         <is>
-          <t>IPATINGA/MG</t>
+          <t>SAO LUIS</t>
         </is>
       </c>
       <c r="AF152" t="inlineStr">
         <is>
-          <t>0 - 8 Dias</t>
+          <t>Acima de 12 Dias</t>
         </is>
       </c>
       <c r="AG152" t="inlineStr">
         <is>
-          <t>PARAUAPEBAS</t>
-        </is>
-      </c>
-      <c r="AH152" t="inlineStr"/>
-      <c r="AI152" t="inlineStr"/>
-      <c r="AJ152" t="b">
-        <v>0</v>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AH152" t="inlineStr">
+        <is>
+          <t>VALE SA</t>
+        </is>
+      </c>
+      <c r="AI152" t="inlineStr">
+        <is>
+          <t>VALE SA</t>
+        </is>
+      </c>
+      <c r="AJ152" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>40219</t>
+          <t>40811</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>1194154</v>
+        <v>1328744</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
@@ -22898,16 +23192,16 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>TDV Contagem MG</t>
+          <t>TDV Fortaleza - CE</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>2593</v>
+        <v>27357</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>FRACIONADO</t>
+          <t>LOTACAO</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -22927,7 +23221,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>31260415801747000116550030000025931705512966</t>
+          <t>21260633592510037821550030000273571654701090</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -22937,7 +23231,7 @@
       </c>
       <c r="M153" t="inlineStr"/>
       <c r="N153" t="n">
-        <v>4101104740</v>
+        <v>4512553116</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -22945,40 +23239,36 @@
         </is>
       </c>
       <c r="P153" s="1" t="n">
-        <v>46136</v>
+        <v>46196</v>
       </c>
       <c r="Q153" t="inlineStr"/>
-      <c r="R153" t="inlineStr">
-        <is>
-          <t>SEVEN SUPRIMENTOS INDUSTRIAIS LTDA</t>
-        </is>
-      </c>
+      <c r="R153" t="inlineStr"/>
       <c r="S153" t="inlineStr">
         <is>
-          <t>MANGUEIRA  P/COMPRESSOR PARAGUSO</t>
+          <t>RODA FERVRIA 42POL 252,1MM</t>
         </is>
       </c>
       <c r="T153" t="inlineStr">
         <is>
-          <t>NOTA FISCAL DIVERGENTE</t>
+          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
         </is>
       </c>
       <c r="U153" t="n">
-        <v>300254000</v>
+        <v>300297000</v>
       </c>
       <c r="V153" t="n">
-        <v>6000153276</v>
+        <v>6000180276</v>
       </c>
       <c r="W153" s="1" t="n">
-        <v>46122</v>
+        <v>46190</v>
       </c>
       <c r="X153" t="inlineStr">
         <is>
-          <t>dluz</t>
+          <t>proliveira</t>
         </is>
       </c>
       <c r="Y153" t="n">
-        <v>702.84</v>
+        <v>318009.11</v>
       </c>
       <c r="Z153" t="inlineStr">
         <is>
@@ -22991,55 +23281,57 @@
         </is>
       </c>
       <c r="AB153" t="n">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="AC153" t="inlineStr">
         <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AD153" t="inlineStr">
+        <is>
+          <t>RECUSADO DEVIDO A INCAPACIDADE PARA DESCARGA DO MATERIAL DE FORMA SEGURA. MATERIL CARREGADO SEM ESTAR PALETIZADO, DIRETAMENTE NO ASSOALHO DO VEICULO.</t>
+        </is>
+      </c>
+      <c r="AE153" t="inlineStr">
+        <is>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AF153" t="inlineStr">
+        <is>
+          <t>Acima de 12 Dias</t>
+        </is>
+      </c>
+      <c r="AG153" t="inlineStr">
+        <is>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AH153" t="inlineStr">
+        <is>
+          <t>VALE S A</t>
+        </is>
+      </c>
+      <c r="AI153" t="inlineStr">
+        <is>
+          <t>VALE SA</t>
+        </is>
+      </c>
+      <c r="AJ153" t="inlineStr">
+        <is>
           <t>NÃO</t>
         </is>
-      </c>
-      <c r="AD153" t="inlineStr">
-        <is>
-          <t>NF CONSTA DIVERGENCIA (INAPTA),NECESSARIO REGULARIZACAO DO XML. O FORNECEDOR DEVERA ABRIR CHAMADO NA FERRAMENTA V360</t>
-        </is>
-      </c>
-      <c r="AE153" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AF153" t="inlineStr">
-        <is>
-          <t>Acima de 12 Dias</t>
-        </is>
-      </c>
-      <c r="AG153" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AH153" t="inlineStr">
-        <is>
-          <t>VALE S A</t>
-        </is>
-      </c>
-      <c r="AI153" t="inlineStr">
-        <is>
-          <t>SEVEN SUPRIMENTOS INDUSTRIAIS LTDA</t>
-        </is>
-      </c>
-      <c r="AJ153" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>40547</t>
+          <t>40828</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>392391</v>
+        <v>1328772</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
@@ -23048,16 +23340,16 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>TDV São Luiz - MA</t>
+          <t>TDV Fortaleza - CE</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>33540</v>
+        <v>27356</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>FRACIONADO</t>
+          <t>LOTACAO</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -23077,7 +23369,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>35250500017952000118550010000335401611802796</t>
+          <t>21260633592510037821550030000273561817592450</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -23087,7 +23379,7 @@
       </c>
       <c r="M154" t="inlineStr"/>
       <c r="N154" t="n">
-        <v>4100989446</v>
+        <v>4512553116</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -23095,34 +23387,36 @@
         </is>
       </c>
       <c r="P154" s="1" t="n">
-        <v>46171</v>
+        <v>46197</v>
       </c>
       <c r="Q154" t="inlineStr"/>
-      <c r="R154" t="inlineStr">
-        <is>
-          <t>MOLYGRAFIT INDUSTRIA E COMERCIO LTD</t>
-        </is>
-      </c>
+      <c r="R154" t="inlineStr"/>
       <c r="S154" t="inlineStr">
         <is>
-          <t>SERVIÇO DE TRANSPORTE</t>
+          <t>RODA FERVRIA 42POL 252,1MM</t>
         </is>
       </c>
       <c r="T154" t="inlineStr">
         <is>
-          <t>NOTA FISCAL DIVERGENTE</t>
-        </is>
-      </c>
-      <c r="U154" t="inlineStr"/>
-      <c r="V154" t="inlineStr"/>
-      <c r="W154" t="inlineStr"/>
+          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
+        </is>
+      </c>
+      <c r="U154" t="n">
+        <v>300292000</v>
+      </c>
+      <c r="V154" t="n">
+        <v>6000177916</v>
+      </c>
+      <c r="W154" s="1" t="n">
+        <v>46184</v>
+      </c>
       <c r="X154" t="inlineStr">
         <is>
-          <t>dluz</t>
+          <t>proliveira</t>
         </is>
       </c>
       <c r="Y154" t="n">
-        <v>1029.23</v>
+        <v>289099.19</v>
       </c>
       <c r="Z154" t="inlineStr">
         <is>
@@ -23135,55 +23429,57 @@
         </is>
       </c>
       <c r="AB154" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="AC154" t="inlineStr">
         <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AD154" t="inlineStr">
+        <is>
+          <t>RECUSADO DEVIDO A INCAPACIDADE DO MATERIAL PARA DESCARREGAR COM EMPILHADEIRA</t>
+        </is>
+      </c>
+      <c r="AE154" t="inlineStr">
+        <is>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AF154" t="inlineStr">
+        <is>
+          <t>Acima de 12 Dias</t>
+        </is>
+      </c>
+      <c r="AG154" t="inlineStr">
+        <is>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AH154" t="inlineStr">
+        <is>
+          <t>VALE S A</t>
+        </is>
+      </c>
+      <c r="AI154" t="inlineStr">
+        <is>
+          <t>VALE SA</t>
+        </is>
+      </c>
+      <c r="AJ154" t="inlineStr">
+        <is>
           <t>NÃO</t>
         </is>
-      </c>
-      <c r="AD154" t="inlineStr">
-        <is>
-          <t>FIZEMOS A TENTATIVA DE REENTREGA COM MESMA NF , JUNTO DA NF COMPLEMENTAR (33689) FONFORME TRATATIVAS , POREM NOTA CONTINUA INAPTA.</t>
-        </is>
-      </c>
-      <c r="AE154" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AF154" t="inlineStr">
-        <is>
-          <t>Acima de 12 Dias</t>
-        </is>
-      </c>
-      <c r="AG154" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AH154" t="inlineStr">
-        <is>
-          <t>VALE S A</t>
-        </is>
-      </c>
-      <c r="AI154" t="inlineStr">
-        <is>
-          <t>MOLYGRAFIT INDUSTRIA E COMERCIO LTD</t>
-        </is>
-      </c>
-      <c r="AJ154" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>40810</t>
+          <t>40829</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>1365998</v>
+        <v>1328771</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -23192,16 +23488,16 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>TDV Contagem MG</t>
+          <t>TDV Fortaleza - CE</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>8466</v>
+        <v>27355</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>FRACIONADO</t>
+          <t>LOTACAO</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -23221,7 +23517,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>31260343711951000505550010000084661325509470</t>
+          <t>21260633592510037821550030000273551780304343</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -23230,24 +23526,22 @@
         </is>
       </c>
       <c r="M155" t="inlineStr"/>
-      <c r="N155" t="inlineStr"/>
+      <c r="N155" t="n">
+        <v>4512553116</v>
+      </c>
       <c r="O155" t="inlineStr">
         <is>
           <t>SAO LUIS</t>
         </is>
       </c>
       <c r="P155" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="Q155" t="inlineStr"/>
-      <c r="R155" t="inlineStr">
-        <is>
-          <t>FLSMIDTH INDUSTRIAL SOLUTIONS LTDA</t>
-        </is>
-      </c>
+      <c r="R155" t="inlineStr"/>
       <c r="S155" t="inlineStr">
         <is>
-          <t>PARTES</t>
+          <t>RODA FERVRIA 42POL 252,1MM</t>
         </is>
       </c>
       <c r="T155" t="inlineStr">
@@ -23259,10 +23553,10 @@
         <v>300292000</v>
       </c>
       <c r="V155" t="n">
-        <v>6000181717</v>
+        <v>6000177916</v>
       </c>
       <c r="W155" s="1" t="n">
-        <v>46195</v>
+        <v>46184</v>
       </c>
       <c r="X155" t="inlineStr">
         <is>
@@ -23270,7 +23564,7 @@
         </is>
       </c>
       <c r="Y155" t="n">
-        <v>1281886.36</v>
+        <v>318009.11</v>
       </c>
       <c r="Z155" t="inlineStr">
         <is>
@@ -23283,55 +23577,57 @@
         </is>
       </c>
       <c r="AB155" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AC155" t="inlineStr">
         <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="AD155" t="inlineStr">
+        <is>
+          <t>RECUSADO DEVIDO A INCAPACIDADE DO MATERIAL PARA DESCARREGAR COM EMPILHADEIRA</t>
+        </is>
+      </c>
+      <c r="AE155" t="inlineStr">
+        <is>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AF155" t="inlineStr">
+        <is>
+          <t>Acima de 12 Dias</t>
+        </is>
+      </c>
+      <c r="AG155" t="inlineStr">
+        <is>
+          <t>SAO LUIS</t>
+        </is>
+      </c>
+      <c r="AH155" t="inlineStr">
+        <is>
+          <t>VALE S A</t>
+        </is>
+      </c>
+      <c r="AI155" t="inlineStr">
+        <is>
+          <t>VALE SA</t>
+        </is>
+      </c>
+      <c r="AJ155" t="inlineStr">
+        <is>
           <t>NÃO</t>
         </is>
-      </c>
-      <c r="AD155" t="inlineStr">
-        <is>
-          <t>O FORNECEDOR DEVERA ABRIR CHAMADO NA FERRAMENTA V360</t>
-        </is>
-      </c>
-      <c r="AE155" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AF155" t="inlineStr">
-        <is>
-          <t>Acima de 12 Dias</t>
-        </is>
-      </c>
-      <c r="AG155" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AH155" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AI155" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AJ155" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>40811</t>
+          <t>40835</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>1328744</v>
+        <v>1331164</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
@@ -23340,16 +23636,16 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>TDV Fortaleza - CE</t>
+          <t>TDV Serra- ES</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>27357</v>
+        <v>24102</v>
       </c>
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>LOTACAO</t>
+          <t>FRACIONADO</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -23369,7 +23665,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>21260633592510037821550030000273571654701090</t>
+          <t>32260501595865000100550010000241021803691646</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -23378,22 +23674,24 @@
         </is>
       </c>
       <c r="M156" t="inlineStr"/>
-      <c r="N156" t="n">
-        <v>4512553116</v>
-      </c>
+      <c r="N156" t="inlineStr"/>
       <c r="O156" t="inlineStr">
         <is>
           <t>SAO LUIS</t>
         </is>
       </c>
       <c r="P156" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="Q156" t="inlineStr"/>
-      <c r="R156" t="inlineStr"/>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>CSV LTDA</t>
+        </is>
+      </c>
       <c r="S156" t="inlineStr">
         <is>
-          <t>RODA FERVRIA 42POL 252,1MM</t>
+          <t>BTN003</t>
         </is>
       </c>
       <c r="T156" t="inlineStr">
@@ -23402,13 +23700,13 @@
         </is>
       </c>
       <c r="U156" t="n">
-        <v>300297000</v>
+        <v>300289000</v>
       </c>
       <c r="V156" t="n">
-        <v>6000180276</v>
+        <v>6000178002</v>
       </c>
       <c r="W156" s="1" t="n">
-        <v>46190</v>
+        <v>46184</v>
       </c>
       <c r="X156" t="inlineStr">
         <is>
@@ -23416,7 +23714,7 @@
         </is>
       </c>
       <c r="Y156" t="n">
-        <v>318009.11</v>
+        <v>46150</v>
       </c>
       <c r="Z156" t="inlineStr">
         <is>
@@ -23429,7 +23727,7 @@
         </is>
       </c>
       <c r="AB156" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AC156" t="inlineStr">
         <is>
@@ -23438,7 +23736,7 @@
       </c>
       <c r="AD156" t="inlineStr">
         <is>
-          <t>RECUSADO DEVIDO A INCAPACIDADE PARA DESCARGA DO MATERIAL DE FORMA SEGURA. MATERIL CARREGADO SEM ESTAR PALETIZADO, DIRETAMENTE NO ASSOALHO DO VEICULO.</t>
+          <t>NAO RECEBIDO POR FALTA DA EQUIPE NO LOCAL PARA REALIZAR O DESCARREGAMENTO</t>
         </is>
       </c>
       <c r="AE156" t="inlineStr">
@@ -23466,38 +23764,30 @@
           <t>VALE SA</t>
         </is>
       </c>
-      <c r="AJ156" t="b">
-        <v>0</v>
+      <c r="AJ156" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>40828</t>
-        </is>
-      </c>
-      <c r="B157" t="n">
-        <v>1328772</v>
-      </c>
+          <t>41002</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
       <c r="C157" t="inlineStr">
         <is>
           <t>Devolução</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>TDV Fortaleza - CE</t>
-        </is>
-      </c>
+      <c r="D157" t="inlineStr"/>
       <c r="E157" t="n">
-        <v>27356</v>
+        <v>65592</v>
       </c>
       <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>LOTACAO</t>
-        </is>
-      </c>
+      <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
           <t>PENDENTE</t>
@@ -23515,7 +23805,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>21260633592510037821550030000273561817592450</t>
+          <t>35260759511741000180550010000655921682706407</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
@@ -23524,49 +23814,41 @@
         </is>
       </c>
       <c r="M157" t="inlineStr"/>
-      <c r="N157" t="n">
-        <v>4512553116</v>
-      </c>
+      <c r="N157" t="inlineStr"/>
       <c r="O157" t="inlineStr">
         <is>
           <t>SAO LUIS</t>
         </is>
       </c>
       <c r="P157" s="1" t="n">
-        <v>46197</v>
+        <v>46223</v>
       </c>
       <c r="Q157" t="inlineStr"/>
-      <c r="R157" t="inlineStr"/>
-      <c r="S157" t="inlineStr">
-        <is>
-          <t>RODA FERVRIA 42POL 252,1MM</t>
-        </is>
-      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>ARGA FACIL DE DESCALVADO LTDA</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr"/>
       <c r="T157" t="inlineStr">
         <is>
           <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
         </is>
       </c>
-      <c r="U157" t="n">
-        <v>300292000</v>
-      </c>
-      <c r="V157" t="n">
-        <v>6000177916</v>
-      </c>
-      <c r="W157" s="1" t="n">
-        <v>46184</v>
-      </c>
+      <c r="U157" t="inlineStr"/>
+      <c r="V157" t="inlineStr"/>
+      <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr">
         <is>
           <t>proliveira</t>
         </is>
       </c>
       <c r="Y157" t="n">
-        <v>289099.19</v>
+        <v>5775</v>
       </c>
       <c r="Z157" t="inlineStr">
         <is>
-          <t>Atrasado</t>
+          <t>No Prazo</t>
         </is>
       </c>
       <c r="AA157" t="inlineStr">
@@ -23575,7 +23857,7 @@
         </is>
       </c>
       <c r="AB157" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AC157" t="inlineStr">
         <is>
@@ -23584,7 +23866,7 @@
       </c>
       <c r="AD157" t="inlineStr">
         <is>
-          <t>RECUSADO DEVIDO A INCAPACIDADE DO MATERIAL PARA DESCARREGAR COM EMPILHADEIRA</t>
+          <t>NF DEVOLVIDA DEVIDO O MATERIAL NAO ESTA PALETIZADO</t>
         </is>
       </c>
       <c r="AE157" t="inlineStr">
@@ -23594,7 +23876,7 @@
       </c>
       <c r="AF157" t="inlineStr">
         <is>
-          <t>Acima de 12 Dias</t>
+          <t>0 - 8 Dias</t>
         </is>
       </c>
       <c r="AG157" t="inlineStr">
@@ -23602,432 +23884,12 @@
           <t>SAO LUIS</t>
         </is>
       </c>
-      <c r="AH157" t="inlineStr">
-        <is>
-          <t>VALE S A</t>
-        </is>
-      </c>
-      <c r="AI157" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AJ157" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>40829</t>
-        </is>
-      </c>
-      <c r="B158" t="n">
-        <v>1328771</v>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>Devolução</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>TDV Fortaleza - CE</t>
-        </is>
-      </c>
-      <c r="E158" t="n">
-        <v>27355</v>
-      </c>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>LOTACAO</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>São Luíz - MA</t>
-        </is>
-      </c>
-      <c r="J158" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="K158" t="inlineStr">
-        <is>
-          <t>21260633592510037821550030000273551780304343</t>
-        </is>
-      </c>
-      <c r="L158" t="inlineStr">
-        <is>
-          <t>VALE</t>
-        </is>
-      </c>
-      <c r="M158" t="inlineStr"/>
-      <c r="N158" t="n">
-        <v>4512553116</v>
-      </c>
-      <c r="O158" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="P158" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="Q158" t="inlineStr"/>
-      <c r="R158" t="inlineStr"/>
-      <c r="S158" t="inlineStr">
-        <is>
-          <t>RODA FERVRIA 42POL 252,1MM</t>
-        </is>
-      </c>
-      <c r="T158" t="inlineStr">
-        <is>
-          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
-        </is>
-      </c>
-      <c r="U158" t="n">
-        <v>300292000</v>
-      </c>
-      <c r="V158" t="n">
-        <v>6000177916</v>
-      </c>
-      <c r="W158" s="1" t="n">
-        <v>46184</v>
-      </c>
-      <c r="X158" t="inlineStr">
-        <is>
-          <t>proliveira</t>
-        </is>
-      </c>
-      <c r="Y158" t="n">
-        <v>318009.11</v>
-      </c>
-      <c r="Z158" t="inlineStr">
-        <is>
-          <t>Atrasado</t>
-        </is>
-      </c>
-      <c r="AA158" t="inlineStr">
-        <is>
-          <t>Em Aberto</t>
-        </is>
-      </c>
-      <c r="AB158" t="n">
-        <v>27</v>
-      </c>
-      <c r="AC158" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="AD158" t="inlineStr">
-        <is>
-          <t>RECUSADO DEVIDO A INCAPACIDADE DO MATERIAL PARA DESCARREGAR COM EMPILHADEIRA</t>
-        </is>
-      </c>
-      <c r="AE158" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AF158" t="inlineStr">
-        <is>
-          <t>Acima de 12 Dias</t>
-        </is>
-      </c>
-      <c r="AG158" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AH158" t="inlineStr">
-        <is>
-          <t>VALE S A</t>
-        </is>
-      </c>
-      <c r="AI158" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AJ158" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>40835</t>
-        </is>
-      </c>
-      <c r="B159" t="n">
-        <v>1331164</v>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Devolução</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>TDV Serra- ES</t>
-        </is>
-      </c>
-      <c r="E159" t="n">
-        <v>24102</v>
-      </c>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>FRACIONADO</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>São Luíz - MA</t>
-        </is>
-      </c>
-      <c r="J159" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>32260501595865000100550010000241021803691646</t>
-        </is>
-      </c>
-      <c r="L159" t="inlineStr">
-        <is>
-          <t>VALE</t>
-        </is>
-      </c>
-      <c r="M159" t="inlineStr"/>
-      <c r="N159" t="inlineStr"/>
-      <c r="O159" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="P159" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="Q159" t="inlineStr"/>
-      <c r="R159" t="inlineStr">
-        <is>
-          <t>CSV LTDA</t>
-        </is>
-      </c>
-      <c r="S159" t="inlineStr">
-        <is>
-          <t>BTN003</t>
-        </is>
-      </c>
-      <c r="T159" t="inlineStr">
-        <is>
-          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
-        </is>
-      </c>
-      <c r="U159" t="n">
-        <v>300289000</v>
-      </c>
-      <c r="V159" t="n">
-        <v>6000178002</v>
-      </c>
-      <c r="W159" s="1" t="n">
-        <v>46184</v>
-      </c>
-      <c r="X159" t="inlineStr">
-        <is>
-          <t>proliveira</t>
-        </is>
-      </c>
-      <c r="Y159" t="n">
-        <v>46150</v>
-      </c>
-      <c r="Z159" t="inlineStr">
-        <is>
-          <t>Atrasado</t>
-        </is>
-      </c>
-      <c r="AA159" t="inlineStr">
-        <is>
-          <t>Em Aberto</t>
-        </is>
-      </c>
-      <c r="AB159" t="n">
-        <v>27</v>
-      </c>
-      <c r="AC159" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="AD159" t="inlineStr">
-        <is>
-          <t>NAO RECEBIDO POR FALTA DA EQUIPE NO LOCAL PARA REALIZAR O DESCARREGAMENTO</t>
-        </is>
-      </c>
-      <c r="AE159" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AF159" t="inlineStr">
-        <is>
-          <t>Acima de 12 Dias</t>
-        </is>
-      </c>
-      <c r="AG159" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AH159" t="inlineStr">
-        <is>
-          <t>VALE S A</t>
-        </is>
-      </c>
-      <c r="AI159" t="inlineStr">
-        <is>
-          <t>VALE SA</t>
-        </is>
-      </c>
-      <c r="AJ159" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>41002</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr"/>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>Devolução</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr"/>
-      <c r="E160" t="n">
-        <v>65592</v>
-      </c>
-      <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr"/>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>São Luíz - MA</t>
-        </is>
-      </c>
-      <c r="J160" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="K160" t="inlineStr">
-        <is>
-          <t>35260759511741000180550010000655921682706407</t>
-        </is>
-      </c>
-      <c r="L160" t="inlineStr">
-        <is>
-          <t>VALE</t>
-        </is>
-      </c>
-      <c r="M160" t="inlineStr"/>
-      <c r="N160" t="inlineStr"/>
-      <c r="O160" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="P160" s="1" t="n">
-        <v>46223</v>
-      </c>
-      <c r="Q160" t="inlineStr"/>
-      <c r="R160" t="inlineStr">
-        <is>
-          <t>ARGA FACIL DE DESCALVADO LTDA</t>
-        </is>
-      </c>
-      <c r="S160" t="inlineStr"/>
-      <c r="T160" t="inlineStr">
-        <is>
-          <t>SEM AUTORIZACAO DE RECEBIMENTO</t>
-        </is>
-      </c>
-      <c r="U160" t="inlineStr"/>
-      <c r="V160" t="inlineStr"/>
-      <c r="W160" t="inlineStr"/>
-      <c r="X160" t="inlineStr">
-        <is>
-          <t>proliveira</t>
-        </is>
-      </c>
-      <c r="Y160" t="n">
-        <v>5775</v>
-      </c>
-      <c r="Z160" t="inlineStr">
-        <is>
-          <t>No Prazo</t>
-        </is>
-      </c>
-      <c r="AA160" t="inlineStr">
-        <is>
-          <t>Em Aberto</t>
-        </is>
-      </c>
-      <c r="AB160" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC160" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="AD160" t="inlineStr">
-        <is>
-          <t>NF DEVOLVIDA DEVIDO O MATERIAL NAO ESTA PALETIZADO</t>
-        </is>
-      </c>
-      <c r="AE160" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AF160" t="inlineStr">
-        <is>
-          <t>0 - 8 Dias</t>
-        </is>
-      </c>
-      <c r="AG160" t="inlineStr">
-        <is>
-          <t>SAO LUIS</t>
-        </is>
-      </c>
-      <c r="AH160" t="inlineStr"/>
-      <c r="AI160" t="inlineStr"/>
-      <c r="AJ160" t="b">
-        <v>0</v>
+      <c r="AH157" t="inlineStr"/>
+      <c r="AI157" t="inlineStr"/>
+      <c r="AJ157" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reclassifica 7 'sem cadastro' como MRO=SIM (B.O. da Vale)
- 7 recusas Parauapebas antes '.' agora MRO=SIM (responsabilidade Vale)
- MRO=SIM: 104->111 | pedido: 78->85 coletas / R$ 2,63mi (2.627.277,21)
- Vale reentregou: 25%->23% (26 de 111)
- Categoria 'sem cadastro' removida do deck (donut agora 2 fatias)
- Timeline (Jul 12->19), destinos (Parauapebas 11->18) e base tratada
  atualizados

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PANxrCPXPZu6Z7SQtmhUMy
</commit_message>
<xml_diff>
--- a/apresentacoes/Devolucoes_Vale_tratada.xlsx
+++ b/apresentacoes/Devolucoes_Vale_tratada.xlsx
@@ -21289,7 +21289,7 @@
       </c>
       <c r="AC139" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD139" t="inlineStr">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="AC140" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD140" t="inlineStr">
@@ -21593,7 +21593,7 @@
       </c>
       <c r="AC141" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD141" t="inlineStr">
@@ -21745,7 +21745,7 @@
       </c>
       <c r="AC142" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD142" t="inlineStr">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="AC143" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD143" t="inlineStr">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="AC144" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD144" t="inlineStr">
@@ -22201,7 +22201,7 @@
       </c>
       <c r="AC145" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="AD145" t="inlineStr">

</xml_diff>